<commit_message>
fix type in bps_updated_jan2026
</commit_message>
<xml_diff>
--- a/bps_updated_jan2026.xlsx
+++ b/bps_updated_jan2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pflue\Dropbox\JacksonHole2024\update December 2025\Figures and Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pflue\OneDrive\Documents\GitHub\carolinpflueger_repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895EE485-8BB6-48BC-85CB-3B1B98D88B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1493EA27-6BA3-46C3-B7F5-01CBC678EB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{FE3E0A03-D39D-4F03-808C-19803518227F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" activeTab="4" xr2:uid="{FE3E0A03-D39D-4F03-808C-19803518227F}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="5" r:id="rId1"/>
@@ -84,9 +84,6 @@
   </si>
   <si>
     <t>y10SE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This file updates the main data series of Bauer, Pflueger abd Sunderam "Perceptions of Monetary Policy (2024, QJE) and Bauer, Pflueger, and Sunderam "Changing Perceptions and Post-Pandemic Monetary Policy (2024, Jackson Hole Proceedings). </t>
   </si>
   <si>
     <r>
@@ -188,6 +185,9 @@
   </si>
   <si>
     <t xml:space="preserve">The last month included in the update is the December 2025 Blue Chip of Financial Forecasters survey and and 1/13/2026 CPI release. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">This file updates the main data series of Bauer, Pflueger and Sunderam "Perceptions of Monetary Policy (2024, QJE) and Bauer, Pflueger, and Sunderam "Changing Perceptions and Post-Pandemic Monetary Policy (2024, Jackson Hole Proceedings). </t>
   </si>
 </sst>
 </file>
@@ -1219,7 +1219,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -1239,27 +1239,27 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -29894,7 +29894,7 @@
         <v>11</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -30549,7 +30549,7 @@
         <v>0.14135204160190001</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">

</xml_diff>